<commit_message>
v11 fish import: bg aliases, treatment loaders, legacy genotype seeding, tank labels
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/genetic_backgrounds.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/genetic_backgrounds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD93EEAB-CCD8-414D-B1CB-972963E0D997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BB63B5A-8804-6948-8F5D-35AC87AC1583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5780" yWindow="14460" windowWidth="27640" windowHeight="16680" xr2:uid="{8D131FA6-D077-A547-B95D-DA88D2CA6F42}"/>
+    <workbookView xWindow="23040" yWindow="18160" windowWidth="27640" windowHeight="16680" xr2:uid="{8D131FA6-D077-A547-B95D-DA88D2CA6F42}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>name</t>
   </si>
@@ -44,13 +44,22 @@
     <t>casper</t>
   </si>
   <si>
-    <t>pIGLET 14a</t>
-  </si>
-  <si>
     <t>alias</t>
   </si>
   <si>
     <t>casper/rnf</t>
+  </si>
+  <si>
+    <t>piglet24b</t>
+  </si>
+  <si>
+    <t>pIGLET14a</t>
+  </si>
+  <si>
+    <t>casper_ab</t>
+  </si>
+  <si>
+    <t>casper/AB</t>
   </si>
 </sst>
 </file>
@@ -422,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F901BCB-D046-6843-A50F-F9BA5949AFAB}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -430,7 +439,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -438,12 +447,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix legacy pipelines + slug-infer gating; clutch background migration and loader
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/genetic_backgrounds.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/genetic_backgrounds.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BB63B5A-8804-6948-8F5D-35AC87AC1583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C99DCA-1A6B-3F4E-9210-C3E7F2D06F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23040" yWindow="18160" windowWidth="27640" windowHeight="16680" xr2:uid="{8D131FA6-D077-A547-B95D-DA88D2CA6F42}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>name</t>
   </si>
@@ -56,10 +56,7 @@
     <t>pIGLET14a</t>
   </si>
   <si>
-    <t>casper_ab</t>
-  </si>
-  <si>
-    <t>casper/AB</t>
+    <t>AB</t>
   </si>
 </sst>
 </file>
@@ -452,15 +449,12 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>